<commit_message>
feat: complete quality engineering initiative
</commit_message>
<xml_diff>
--- a/reports/xlsx/execution_results.xlsx
+++ b/reports/xlsx/execution_results.xlsx
@@ -437,7 +437,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-21T13:18:45</t>
+          <t>2026-09-25T11:42:14</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -482,7 +482,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>22.651</v>
+        <v>13.926</v>
       </c>
     </row>
     <row r="10">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>31.033</v>
+        <v>326.976</v>
       </c>
     </row>
     <row r="11">
@@ -532,7 +532,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -543,7 +543,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Poor</t>
+          <t>Excellent</t>
         </is>
       </c>
     </row>
@@ -558,7 +558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -651,26 +651,26 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>TC_15</t>
+          <t>TC_01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TC_15 - Concurrent Transaction Assessment</t>
+          <t>TC_01 - Criar Conta</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Quality Engineering - Avaliação de Qualidade</t>
+          <t>Cadastro de contas</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>22.651</v>
+        <v>7.66</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -684,55 +684,1308 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Fluxo concluído com sucesso</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>evidencias\geral\TC_15</t>
+          <t>evidencias\cadastro\TC_01</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>videos/TC_15_-_Concurrent_Transaction_Assessment/video.webm</t>
+          <t>videos/TC_01_-_Criar_Conta/video.webm</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>https://bugbank.netlify.app/home</t>
+          <t>https://bugbank.netlify.app/</t>
         </is>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>123</v>
+        <v>20</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-21T13:18:43</t>
+          <t>2026-09-25T11:37:01</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/01_inicio.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/02_acionar_a_confirma_o_da_transfer_ncia_5_vezes_em_r_pida_suce.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/02_existe_uma_conta_receptora_v_lida.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/02_o_saldo_do_remetente_dever_ter_sido_debitado_exatamente_uma.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/02_preencher_uma_transfer_ncia_v_lida_de_50_reais.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/02_que_o_usu_rio_remetente_est_autenticado_com_saldo_inicial_su.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/failed.png
-videos/TC_15_-_Concurrent_Transaction_Assessment/screenshots/falha_o_saldo_do_remetente_dever_ter_sido_debitado_exatamente_uma.png</t>
+          <t>videos/TC_01_-_Criar_Conta/screenshots/01_inicio.png
+videos/TC_01_-_Criar_Conta/screenshots/02_a_conta_dever_ser_criada_com_sucesso.png
+videos/TC_01_-_Criar_Conta/screenshots/02_clicar_em_Cadastrar.png
+videos/TC_01_-_Criar_Conta/screenshots/02_informar_nome_e-mail_senha_e_confirma_o_de_senha_v_lidos.png
+videos/TC_01_-_Criar_Conta/screenshots/02_que_o_usu_rio_est_na_tela_de_cadastro.png
+videos/TC_01_-_Criar_Conta/screenshots/03_sucesso.png</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>videos/TC_15_-_Concurrent_Transaction_Assessment/execution.log</t>
+          <t>videos/TC_01_-_Criar_Conta/execution.log</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>videos/TC_15_-_Concurrent_Transaction_Assessment/html/page_source.html</t>
+          <t>videos/TC_01_-_Criar_Conta/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TC_03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TC_03 - Criar Conta com Saldo Inicial</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cadastro de contas</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>7.449</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>evidencias\cadastro\TC_03</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/video.webm</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>20</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:37:15</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/01_inicio.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/02_a_conta_dever_possuir_saldo_inicial_dispon_vel.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/02_a_conta_dever_ser_criada_com_sucesso.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/02_clicar_em_Cadastrar.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/02_informar_nome_e-mail_senha_e_confirma_o_de_senha_v_lidos.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/02_que_o_usu_rio_est_na_tela_de_cadastro.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/02_selecionar_a_op_o_Criar_conta_com_saldo.png
+videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/execution.log</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>videos/TC_03_-_Criar_Conta_com_Saldo_Inicial/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TC_04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TC_04 - Validar Campos Obrigatórios do Cadastro</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Cadastro de contas</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>5.693</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>evidencias\cadastro\TC_04</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/video.webm</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>20</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:37:31</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/01_inicio.png
+videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/02_a_conta_n_o_dever_ser_criada.png
+videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/02_clicar_em_Cadastrar.png
+videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/02_deixar_os_campos_obrigat_rios_em_branco.png
+videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/02_mensagens_de_valida_o_dever_o_ser_apresentadas.png
+videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/02_que_o_usu_rio_est_na_tela_de_cadastro.png
+videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/execution.log</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>videos/TC_04_-_Validar_Campos_Obrigat_rios_do_Cadastro/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>TC_05</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TC_05 - Cadastrar Conta com E-mail Já Utilizado</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Cadastro de contas</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>8.544</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>evidencias\cadastro\TC_05</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/video.webm</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:37:47</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/01_inicio.png
+videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/02_a_conta_n_o_dever_ser_criada.png
+videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/02_o_sistema_dever_exibir_uma_mensagem_de_erro.png
+videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/02_o_usu_rio_tentar_criar_uma_nova_conta_utilizando_o_mesmo_e-m.png
+videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/02_preencher_os_demais_campos_obrigat_rios_corretamente.png
+videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/02_que_existe_uma_conta_cadastrada_com_determinado_e-mail.png
+videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/execution.log</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>videos/TC_05_-_Cadastrar_Conta_com_E-mail_J_Utilizado/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TC_06</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC_06 - Cadastrar Conta com Confirmação de Senha Divergente</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Cadastro de contas</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>evidencias\cadastro\TC_06</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/video.webm</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>20</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:38:01</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/01_inicio.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/02_a_conta_n_o_dever_ser_criada.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/02_clicar_em_Cadastrar.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/02_informar_uma_confirma_o_de_senha_diferente.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/02_informar_uma_senha_v_lida.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/02_o_sistema_dever_exibir_uma_mensagem_de_erro.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/02_que_o_usu_rio_est_na_tela_de_cadastro.png
+videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/execution.log</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>videos/TC_06_-_Cadastrar_Conta_com_Confirma_o_de_Senha_Divergente/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>TC_09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TC_09 - Consultar Saldo da Conta</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Saldo, extrato e sessão</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>7.409</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>evidencias\extrato\TC_09</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>videos/TC_09_-_Consultar_Saldo_da_Conta/video.webm</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/home</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>50</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:38:17</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>videos/TC_09_-_Consultar_Saldo_da_Conta/screenshots/01_inicio.png
+videos/TC_09_-_Consultar_Saldo_da_Conta/screenshots/02_acessar_a_p_gina_inicial_da_conta.png
+videos/TC_09_-_Consultar_Saldo_da_Conta/screenshots/02_o_saldo_dispon_vel_dever_ser_exibido.png
+videos/TC_09_-_Consultar_Saldo_da_Conta/screenshots/02_o_valor_exibido_dever_corresponder_ao_saldo_da_conta.png
+videos/TC_09_-_Consultar_Saldo_da_Conta/screenshots/02_que_o_usu_rio_est_autenticado.png
+videos/TC_09_-_Consultar_Saldo_da_Conta/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>videos/TC_09_-_Consultar_Saldo_da_Conta/execution.log</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>videos/TC_09_-_Consultar_Saldo_da_Conta/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TC_12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TC_12 - Fluxo E2E Completo de Transferência, Extrato, Saldo e Logout</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Saldo, extrato e sessão</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>24.659</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>evidencias\extrato\TC_12</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/video.webm</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>208</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:38:49</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/01_inicio.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_acessar_seu_extrato.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_consultar_seu_saldo.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_dever_retornar_para_a_tela_de_login.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_dever_visualizar_o_recebimento_da_transfer_ncia.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_dever_visualizar_o_registro_da_transfer_ncia_enviada.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_o_saldo_dever_refletir_o_cr_dito_recebido.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_o_saldo_dever_refletir_o_d_bito_da_transfer_ncia.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_o_usu_rio_A_realizar_login.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_o_usu_rio_B_realizar_login.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_que_existe_uma_transfer_ncia_realizada_entre_o_usu_rio_A_e_o.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/02_realizar_logout.png
+videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/execution.log</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>videos/TC_12_-_Fluxo_E2E_Completo_de_Transfer_ncia_Extrato_Saldo_e_Logout/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TC_02</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TC_02 - Acessar a Conta</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Autenticação</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>8.885999999999999</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>evidencias\login\TC_02</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>videos/TC_02_-_Acessar_a_Conta/video.webm</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/home</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>50</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:39:07</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>videos/TC_02_-_Acessar_a_Conta/screenshots/01_inicio.png
+videos/TC_02_-_Acessar_a_Conta/screenshots/02_clicar_em_Acessar.png
+videos/TC_02_-_Acessar_a_Conta/screenshots/02_informar_uma_senha_v_lida.png
+videos/TC_02_-_Acessar_a_Conta/screenshots/02_o_usu_rio_dever_ser_autenticado_com_sucesso.png
+videos/TC_02_-_Acessar_a_Conta/screenshots/02_o_usu_rio_informar_um_e-mail_v_lido.png
+videos/TC_02_-_Acessar_a_Conta/screenshots/02_que_existe_uma_conta_cadastrada.png
+videos/TC_02_-_Acessar_a_Conta/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>videos/TC_02_-_Acessar_a_Conta/execution.log</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>videos/TC_02_-_Acessar_a_Conta/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TC_07</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TC_07 - Realizar Login com Senha Inválida</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Autenticação</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>8.582000000000001</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>evidencias\login\TC_07</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/video.webm</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>40</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:39:22</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/01_inicio.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/02_clicar_em_Acessar.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/02_informar_uma_senha_inv_lida.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/02_o_sistema_dever_exibir_uma_mensagem_de_autentica_o_inv_lida.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/02_o_usu_rio_informar_um_e-mail_v_lido.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/02_o_usu_rio_n_o_dever_ser_autenticado.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/02_que_existe_uma_conta_cadastrada.png
+videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/execution.log</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>videos/TC_07_-_Realizar_Login_com_Senha_Inv_lida/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TC_08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TC_08 - Realizar Logout da Aplicação</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Autenticação</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>7.754</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>evidencias\login\TC_08</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>videos/TC_08_-_Realizar_Logout_da_Aplica_o/video.webm</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>50</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:39:36</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>videos/TC_08_-_Realizar_Logout_da_Aplica_o/screenshots/01_inicio.png
+videos/TC_08_-_Realizar_Logout_da_Aplica_o/screenshots/02_a_sess_o_dever_ser_encerrada.png
+videos/TC_08_-_Realizar_Logout_da_Aplica_o/screenshots/02_clicar_na_op_o_de_logout.png
+videos/TC_08_-_Realizar_Logout_da_Aplica_o/screenshots/02_o_usu_rio_dever_ser_redirecionado_para_a_tela_de_login.png
+videos/TC_08_-_Realizar_Logout_da_Aplica_o/screenshots/02_que_o_usu_rio_est_autenticado.png
+videos/TC_08_-_Realizar_Logout_da_Aplica_o/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>videos/TC_08_-_Realizar_Logout_da_Aplica_o/execution.log</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>videos/TC_08_-_Realizar_Logout_da_Aplica_o/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TC_13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TC_13 - Financial Reconciliation Assessment</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Quality Engineering - Avaliação de Qualidade</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>50.555</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>evidencias\geral\TC_13</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>videos/TC_13_-_Financial_Reconciliation_Assessment/video.webm</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/bank-statement</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>622</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:40:33</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/01_inicio.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_a_conta_A_transferir_300_reais_para_a_conta_B.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_a_conta_B_possui_saldo_inicial.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_a_conta_B_transferir_100_reais_para_a_conta_C.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_a_conta_C_n_o_possui_saldo_inicial.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_a_transfer_ncia_da_conta_A_dever_ser_conclu_da_com_sucesso.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_a_transfer_ncia_da_conta_B_dever_ser_conclu_da_com_sucesso.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_extrato_da_conta_A_dever_conter_um_nico_d_bito_de_300.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_extrato_da_conta_B_dever_conter_exatamente_um_cr_dito_de_3.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_extrato_da_conta_C_dever_conter_um_nico_cr_dito_de_100.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_saldo_final_da_conta_A_dever_ser_o_inicial_menos_300.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_saldo_final_da_conta_B_dever_ser_o_inicial_mais_300_menos.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_saldo_final_da_conta_C_dever_ser_100.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_o_total_financeiro_do_sistema_dever_estar_reconciliado.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/02_que_a_conta_A_est_autenticada_com_saldo_inicial.png
+videos/TC_13_-_Financial_Reconciliation_Assessment/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>videos/TC_13_-_Financial_Reconciliation_Assessment/execution.log</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>videos/TC_13_-_Financial_Reconciliation_Assessment/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>TC_14</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TC_14 - Session Integrity Assessment</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Quality Engineering - Avaliação de Qualidade</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>15.909</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>evidencias\geral\TC_14</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>videos/TC_14_-_Session_Integrity_Assessment/video.webm</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>126</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:41:00</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>videos/TC_14_-_Session_Integrity_Assessment/screenshots/01_inicio.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_a_sess_o_dever_permanecer_encerrada.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_a_sess_o_dever_ser_encerrada.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_atualizar_a_p_gina.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_clicar_na_op_o_de_logout.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_o_acesso_rea_protegida_dever_permanecer_bloqueado.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_o_acesso_rea_protegida_dever_ser_bloqueado.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_o_usu_rio_dever_ser_redirecionado_para_a_tela_de_login.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_pressionar_o_bot_o_voltar_do_navegador.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_que_o_usu_rio_est_autenticado.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/02_tentar_acessar_diretamente_a_URL_da_rea_logada.png
+videos/TC_14_-_Session_Integrity_Assessment/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>videos/TC_14_-_Session_Integrity_Assessment/execution.log</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>videos/TC_14_-_Session_Integrity_Assessment/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TC_16</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TC_16 - Data Persistence Assessment</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Quality Engineering - Avaliação de Qualidade</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>22.468</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>evidencias\geral\TC_16</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>videos/TC_16_-_Data_Persistence_Assessment/video.webm</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/bank-statement</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>162</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:41:30</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>videos/TC_16_-_Data_Persistence_Assessment/screenshots/01_inicio.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_a_transfer_ncia_dever_ser_conclu_da_com_sucesso.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_as_movimenta_es_do_extrato_dever_o_estar_preservadas.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_existe_uma_conta_destinat_ria_v_lida_para_transfer_ncia.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_o_saldo_anterior_dever_estar_preservado.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_o_saldo_do_usu_rio_A_dever_ser_atualizado_com_o_d_bito.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_o_usu_rio_A_realizar_login_novamente.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_o_usu_rio_A_realizar_uma_transfer_ncia_de_valor_v_lido.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_que_o_usu_rio_A_est_autenticado_com_saldo_inicial.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_realizar_logout_da_conta.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/02_registrar_o_extrato_da_conta.png
+videos/TC_16_-_Data_Persistence_Assessment/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>videos/TC_16_-_Data_Persistence_Assessment/execution.log</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>videos/TC_16_-_Data_Persistence_Assessment/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>TC_10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TC_10 - Realizar Transferência sem Saldo Suficiente</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Transferências</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>12.073</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>evidencias\transferencia\TC_10</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/video.webm</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/transfer</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>71</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:41:48</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/01_inicio.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_a_transfer_ncia_n_o_dever_ser_realizada.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_confirmar_a_transfer_ncia.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_informar_um_valor_superior_ao_saldo_dispon_vel.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_informar_uma_conta_destinat_ria_v_lida.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_o_saldo_da_conta_dever_permanecer_inalterado.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_o_sistema_dever_exibir_uma_mensagem_de_saldo_insuficiente.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_possui_saldo_insuficiente_para_realizar_uma_transfer_ncia.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/02_que_o_usu_rio_est_autenticado.png
+videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/execution.log</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>videos/TC_10_-_Realizar_Transfer_ncia_sem_Saldo_Suficiente/html/page_source.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TC_11</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TC_11 - Fluxo E2E de Cadastro, Login e Transferência entre Contas</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Transferências</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>14.923</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Faker / dados isolados por cenário</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Fluxo BDD concluído conforme a feature</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Fluxo concluído com sucesso</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>evidencias\transferencia\TC_11</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/video.webm</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>https://bugbank.netlify.app/home</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>98</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-09-25T11:42:10</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/01_inicio.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_a_conta_dever_ser_criada_com_sucesso.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_a_segunda_conta_dever_ser_criada_com_sucesso.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_a_transfer_ncia_dever_ser_realizada_com_sucesso.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_acessar_a_funcionalidade_de_transfer_ncia.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_confirmar_a_opera_o.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_criar_uma_conta_com_saldo_inicial.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_criar_uma_segunda_conta_v_lida.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_informar_os_dados_da_conta_do_usu_rio_B.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_informar_um_valor_v_lido.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_o_saldo_do_usu_rio_A_dever_ser_atualizado.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_o_usu_rio_A_realizar_login.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_que_o_usu_rio_A_est_na_tela_de_cadastro.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/02_que_o_usu_rio_B_est_na_tela_de_cadastro.png
+videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/screenshots/03_sucesso.png</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/execution.log</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>videos/TC_11_-_Fluxo_E2E_de_Cadastro_Login_e_Transfer_ncia_entre_Contas/html/page_source.html</t>
         </is>
       </c>
     </row>

</xml_diff>